<commit_message>
feat: melhorias em admin, usuarios e enquadramento CNAE
</commit_message>
<xml_diff>
--- a/CALCULADORA SIMPLES.xlsx
+++ b/CALCULADORA SIMPLES.xlsx
@@ -5,18 +5,19 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Documents\Guildahub plataforma\simples nacional\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\PLANILHAS DO SIMPLES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1A6C6AA-DC5E-45C5-809F-59597D8E27C5}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E99FD42C-EB8F-4EF3-8C1F-619AFA2D0B3E}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{7486B403-3960-476F-A77B-052D7FF51657}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" activeTab="4" xr2:uid="{7486B403-3960-476F-A77B-052D7FF51657}"/>
   </bookViews>
   <sheets>
     <sheet name="ANEXO I" sheetId="1" r:id="rId1"/>
     <sheet name="ANEXO II" sheetId="2" r:id="rId2"/>
     <sheet name="ANEXO III" sheetId="3" r:id="rId3"/>
     <sheet name="ANEXO IV" sheetId="4" r:id="rId4"/>
+    <sheet name="ANEXO V" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="70">
   <si>
     <t>RBT12</t>
   </si>
@@ -1209,7 +1210,7 @@
         <v>0</v>
       </c>
       <c r="F2" s="6">
-        <v>1170000</v>
+        <v>1900000</v>
       </c>
       <c r="I2" s="49" t="s">
         <v>3</v>
@@ -1310,7 +1311,7 @@
       </c>
       <c r="F6" s="62">
         <f>IF(F2&lt;=180000,K3,IF(AND(F2&gt;=180000.01,F2&lt;=360000),K4,IF(AND(F2&gt;=360000.01,F2&lt;=720000),K5,IF(AND(F2&gt;=720000.01,F2&lt;=1800000),K6,IF(AND(F2&gt;=1800000.01,F2&lt;=3600000),K7,IF(AND(F2&gt;=3600000.01,F2&lt;=4800000),K8,0))))))</f>
-        <v>0.107</v>
+        <v>0.14299999999999999</v>
       </c>
       <c r="I6" s="8" t="s">
         <v>13</v>
@@ -1382,7 +1383,7 @@
       </c>
       <c r="F9" s="51">
         <f>IF(F6=K3,0,IF(F6=K4,L4,IF(F6=K5,L5,IF(F6=K6,L6,IF(F6=K7,L7,IF(F6=K8,L8,0))))))</f>
-        <v>22500</v>
+        <v>87300</v>
       </c>
     </row>
     <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1425,7 +1426,7 @@
       <c r="I12" s="12"/>
       <c r="J12" s="56">
         <f>(((F2*F6)-F9)/F2)</f>
-        <v>8.7769230769230766E-2</v>
+        <v>9.7052631578947363E-2</v>
       </c>
     </row>
     <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1464,7 +1465,7 @@
       </c>
       <c r="F15" s="45">
         <f>F3*J12</f>
-        <v>17553.846153846152</v>
+        <v>19410.526315789473</v>
       </c>
       <c r="G15" s="47"/>
     </row>
@@ -1495,7 +1496,7 @@
       <c r="G18" s="44"/>
       <c r="J18" s="34" t="str">
         <f>IF(F6=K6,I6,IF(F6=K3,I3,IF(F6=K4,I4,IF(F6=K5,I5,IF(F6=K7,I7,IF(F6=K8,I8,0))))))</f>
-        <v>4ª Faixa</v>
+        <v>5ª Faixa</v>
       </c>
       <c r="K18" s="37" t="s">
         <v>66</v>
@@ -1530,12 +1531,12 @@
       </c>
       <c r="K19" s="36">
         <f>IF($J$18=$A$20,$J$12*$B$20,IF($J$18=$A$21,$J$12*$B$21,IF($J$18=$A$22,$J$12*$B$22,IF($J$18=$A$23,$J$12*$B$23,IF($J$18=$A$24,$J$12*$B$24,0)))))</f>
-        <v>4.8273076923076924E-3</v>
+        <v>5.3378947368421048E-3</v>
       </c>
       <c r="L19" s="36"/>
       <c r="M19" s="29">
         <f>$F$3*K19</f>
-        <v>965.46153846153845</v>
+        <v>1067.578947368421</v>
       </c>
       <c r="N19" s="23"/>
       <c r="O19" s="22"/>
@@ -1567,12 +1568,12 @@
       </c>
       <c r="K20" s="36">
         <f>IF($J$18=$A$20,$J$12*$C$20,IF($J$18=$A$21,$J$12*$C$21,IF($J$18=$A$22,$J$12*$C$22,IF($J$18=$A$23,$J$12*$C$23,IF($J$18=$A$24,$J$12*$C$24,0)))))</f>
-        <v>3.0719230769230771E-3</v>
+        <v>3.3968421052631582E-3</v>
       </c>
       <c r="L20" s="36"/>
       <c r="M20" s="29">
         <f t="shared" ref="M20:M24" si="0">$F$3*K20</f>
-        <v>614.38461538461547</v>
+        <v>679.36842105263167</v>
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.25">
@@ -1602,12 +1603,12 @@
       </c>
       <c r="K21" s="36">
         <f>IF($J$18=$A$20,$J$12*$D$20,IF($J$18=$A$21,$J$12*$D$21,IF($J$18=$A$22,$J$12*$D$22,IF($J$18=$A$23,$J$12*$D$23,IF($J$18=$A$24,$J$12*$D$24,0)))))</f>
-        <v>1.11818E-2</v>
+        <v>1.2364505263157896E-2</v>
       </c>
       <c r="L21" s="36"/>
       <c r="M21" s="29">
         <f t="shared" si="0"/>
-        <v>2236.36</v>
+        <v>2472.9010526315792</v>
       </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.25">
@@ -1637,12 +1638,12 @@
       </c>
       <c r="K22" s="36">
         <f>IF($J$18=$A$20,$J$12*$E$20,IF($J$18=$A$21,$J$12*$E$21,IF($J$18=$A$22,$J$12*$E$22,IF($J$18=$A$23,$J$12*$E$23,IF($J$18=$A$24,$J$12*$E$24,0)))))</f>
-        <v>2.4224307692307691E-3</v>
+        <v>2.6786526315789472E-3</v>
       </c>
       <c r="L22" s="36"/>
       <c r="M22" s="29">
         <f t="shared" si="0"/>
-        <v>484.4861538461538</v>
+        <v>535.73052631578946</v>
       </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.25">
@@ -1672,12 +1673,12 @@
       </c>
       <c r="K23" s="36">
         <f>IF($J$18=$A$20,$J$12*$F$20,IF($J$18=$A$21,$J$12*$F$21,IF($J$18=$A$22,$J$12*$F$22,IF($J$18=$A$23,$J$12*$F$23,IF($J$18=$A$24,$J$12*$F$24,0)))))</f>
-        <v>3.6863076923076922E-2</v>
+        <v>4.0762105263157891E-2</v>
       </c>
       <c r="L23" s="36"/>
       <c r="M23" s="29">
         <f t="shared" si="0"/>
-        <v>7372.6153846153848</v>
+        <v>8152.4210526315783</v>
       </c>
     </row>
     <row r="24" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1707,12 +1708,12 @@
       </c>
       <c r="K24" s="39">
         <f>IF($J$18=$A$20,$J$12*$G$20,IF($J$18=$A$21,$J$12*$G$21,IF($J$18=$A$22,$J$12*$G$22,IF($J$18=$A$23,$J$12*$G$23,IF($J$18=$A$24,$J$12*$G$24,0)))))</f>
-        <v>2.9402692307692307E-2</v>
+        <v>3.2512631578947369E-2</v>
       </c>
       <c r="L24" s="39"/>
       <c r="M24" s="31">
         <f t="shared" si="0"/>
-        <v>5880.538461538461</v>
+        <v>6502.5263157894742</v>
       </c>
     </row>
     <row r="25" spans="1:15" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1742,12 +1743,12 @@
       </c>
       <c r="K25" s="38">
         <f>SUM(K19:L24)</f>
-        <v>8.7769230769230766E-2</v>
+        <v>9.7052631578947363E-2</v>
       </c>
       <c r="L25" s="38"/>
       <c r="M25" s="33">
         <f>SUM(M19:M24)</f>
-        <v>17553.846153846152</v>
+        <v>19410.526315789473</v>
       </c>
     </row>
   </sheetData>
@@ -3683,4 +3684,603 @@
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23F678D6-1437-4843-BF31-DA48CD2FC2C1}">
+  <dimension ref="A1:M26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5703125" customWidth="1"/>
+    <col min="6" max="6" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="7.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="26.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="7.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" s="6">
+        <f>C15</f>
+        <v>1170000</v>
+      </c>
+      <c r="I2" s="49" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="50"/>
+      <c r="K2" s="7" t="s">
+        <v>4</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="3">
+        <v>1</v>
+      </c>
+      <c r="C3" s="13">
+        <v>0</v>
+      </c>
+      <c r="E3" s="58" t="s">
+        <v>1</v>
+      </c>
+      <c r="F3" s="60">
+        <v>20000</v>
+      </c>
+      <c r="I3" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="K3" s="17">
+        <v>0.155</v>
+      </c>
+      <c r="L3" s="16" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B4" s="4">
+        <v>2</v>
+      </c>
+      <c r="C4" s="14">
+        <v>195000</v>
+      </c>
+      <c r="E4" s="59"/>
+      <c r="F4" s="61"/>
+      <c r="I4" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="J4" s="16" t="s">
+        <v>10</v>
+      </c>
+      <c r="K4" s="17">
+        <v>0.18</v>
+      </c>
+      <c r="L4" s="18">
+        <v>4500</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>27</v>
+      </c>
+      <c r="B5" s="4">
+        <v>3</v>
+      </c>
+      <c r="C5" s="14"/>
+      <c r="I5" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" s="16" t="s">
+        <v>12</v>
+      </c>
+      <c r="K5" s="17">
+        <v>0.19500000000000001</v>
+      </c>
+      <c r="L5" s="18">
+        <v>9900</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>28</v>
+      </c>
+      <c r="B6" s="4">
+        <v>4</v>
+      </c>
+      <c r="C6" s="14"/>
+      <c r="E6" s="58" t="s">
+        <v>2</v>
+      </c>
+      <c r="F6" s="62">
+        <f>IF(F2&lt;=180000,K3,IF(AND(F2&gt;=180000.01,F2&lt;=360000),K4,IF(AND(F2&gt;=360000.01,F2&lt;=720000),K5,IF(AND(F2&gt;=720000.01,F2&lt;=1800000),K6,IF(AND(F2&gt;=1800000.01,F2&lt;=3600000),K7,IF(AND(F2&gt;=3600000.01,F2&lt;=4800000),K8,0))))))</f>
+        <v>0.20499999999999999</v>
+      </c>
+      <c r="I6" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="J6" s="16" t="s">
+        <v>14</v>
+      </c>
+      <c r="K6" s="17">
+        <v>0.20499999999999999</v>
+      </c>
+      <c r="L6" s="18">
+        <v>17100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>29</v>
+      </c>
+      <c r="B7" s="4">
+        <v>5</v>
+      </c>
+      <c r="C7" s="14"/>
+      <c r="E7" s="59"/>
+      <c r="F7" s="63"/>
+      <c r="I7" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="J7" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="K7" s="17">
+        <v>0.23</v>
+      </c>
+      <c r="L7" s="18">
+        <v>62100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>30</v>
+      </c>
+      <c r="B8" s="4">
+        <v>6</v>
+      </c>
+      <c r="C8" s="14"/>
+      <c r="I8" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="J8" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="K8" s="17">
+        <v>0.30499999999999999</v>
+      </c>
+      <c r="L8" s="18">
+        <v>540000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="4">
+        <v>7</v>
+      </c>
+      <c r="C9" s="14"/>
+      <c r="E9" s="58" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" s="51">
+        <f>IF(F6=K3,0,IF(F6=K4,L4,IF(F6=K5,L5,IF(F6=K6,L6,IF(F6=K7,L7,IF(F6=K8,L8,0))))))</f>
+        <v>17100</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
+        <v>32</v>
+      </c>
+      <c r="B10" s="4">
+        <v>8</v>
+      </c>
+      <c r="C10" s="14"/>
+      <c r="E10" s="59"/>
+      <c r="F10" s="52"/>
+    </row>
+    <row r="11" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
+        <v>33</v>
+      </c>
+      <c r="B11" s="4">
+        <v>9</v>
+      </c>
+      <c r="C11" s="14"/>
+      <c r="J11" s="11"/>
+    </row>
+    <row r="12" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" s="4">
+        <v>10</v>
+      </c>
+      <c r="C12" s="14"/>
+      <c r="E12" s="53" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+      <c r="I12" s="12"/>
+      <c r="J12" s="51">
+        <f>(((F2*F6)-F9)/F2)</f>
+        <v>0.19038461538461537</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" s="4">
+        <v>11</v>
+      </c>
+      <c r="C13" s="14"/>
+      <c r="E13" s="54"/>
+      <c r="F13" s="55" t="s">
+        <v>0</v>
+      </c>
+      <c r="G13" s="55"/>
+      <c r="H13" s="55"/>
+      <c r="I13" s="55"/>
+      <c r="J13" s="52"/>
+    </row>
+    <row r="14" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>36</v>
+      </c>
+      <c r="B14" s="5">
+        <v>12</v>
+      </c>
+      <c r="C14" s="15"/>
+    </row>
+    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="C15">
+        <f>(12*SUM(C3:C14))/COUNTA(C3:C14)</f>
+        <v>1170000</v>
+      </c>
+      <c r="E15" s="45" t="s">
+        <v>22</v>
+      </c>
+      <c r="F15" s="45">
+        <f>F3*J12</f>
+        <v>3807.6923076923076</v>
+      </c>
+      <c r="G15" s="47"/>
+    </row>
+    <row r="16" spans="1:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="E16" s="46"/>
+      <c r="F16" s="46"/>
+      <c r="G16" s="48"/>
+    </row>
+    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="J17" s="67" t="s">
+        <v>69</v>
+      </c>
+      <c r="K17" s="68"/>
+      <c r="L17" s="68"/>
+      <c r="M17" s="69"/>
+    </row>
+    <row r="18" spans="1:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="40" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="42" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="43"/>
+      <c r="D18" s="43"/>
+      <c r="E18" s="43"/>
+      <c r="F18" s="43"/>
+      <c r="G18" s="43"/>
+      <c r="J18" s="27" t="str">
+        <f>IF(F6=K6,I6,IF(F6=K3,I3,IF(F6=K4,I4,IF(F6=K5,I5,IF(F6=K7,I7,IF(F6=K8,I8,0))))))</f>
+        <v>4ª Faixa</v>
+      </c>
+      <c r="K18" s="72" t="s">
+        <v>66</v>
+      </c>
+      <c r="L18" s="72"/>
+      <c r="M18" s="28" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A19" s="41"/>
+      <c r="B19" s="26" t="s">
+        <v>39</v>
+      </c>
+      <c r="C19" s="19" t="s">
+        <v>40</v>
+      </c>
+      <c r="D19" s="19" t="s">
+        <v>41</v>
+      </c>
+      <c r="E19" s="19" t="s">
+        <v>42</v>
+      </c>
+      <c r="F19" s="19" t="s">
+        <v>43</v>
+      </c>
+      <c r="G19" s="19" t="s">
+        <v>46</v>
+      </c>
+      <c r="J19" s="27" t="s">
+        <v>39</v>
+      </c>
+      <c r="K19" s="36">
+        <f>IF($J$18=$A$20,$J$12*$B$20,IF($J$18=$A$21,$J$12*$B$21,IF($J$18=$A$22,$J$12*$B$22,IF($J$18=$A$23,$J$12*$B$23,IF($J$18=$A$24,$J$12*$B$24,0)))))</f>
+        <v>3.9980769230769229E-2</v>
+      </c>
+      <c r="L19" s="36"/>
+      <c r="M19" s="29">
+        <f>$F$3*K19</f>
+        <v>799.61538461538464</v>
+      </c>
+    </row>
+    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A20" s="16" t="s">
+        <v>6</v>
+      </c>
+      <c r="B20" s="17">
+        <v>0.25</v>
+      </c>
+      <c r="C20" s="17">
+        <v>0.15</v>
+      </c>
+      <c r="D20" s="17">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="E20" s="17">
+        <v>3.0499999999999999E-2</v>
+      </c>
+      <c r="F20" s="17">
+        <v>0.28849999999999998</v>
+      </c>
+      <c r="G20" s="17">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="J20" s="27" t="s">
+        <v>40</v>
+      </c>
+      <c r="K20" s="36">
+        <f>IF($J$18=$A$20,$J$12*$C$20,IF($J$18=$A$21,$J$12*$C$21,IF($J$18=$A$22,$J$12*$C$22,IF($J$18=$A$23,$J$12*$C$23,IF($J$18=$A$24,$J$12*$C$24,0)))))</f>
+        <v>2.8557692307692305E-2</v>
+      </c>
+      <c r="L20" s="36"/>
+      <c r="M20" s="29">
+        <f t="shared" ref="M20:M24" si="0">$F$3*K20</f>
+        <v>571.15384615384608</v>
+      </c>
+    </row>
+    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A21" s="16" t="s">
+        <v>9</v>
+      </c>
+      <c r="B21" s="17">
+        <v>0.23</v>
+      </c>
+      <c r="C21" s="17">
+        <v>0.15</v>
+      </c>
+      <c r="D21" s="17">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="E21" s="17">
+        <v>3.0499999999999999E-2</v>
+      </c>
+      <c r="F21" s="17">
+        <v>0.27850000000000003</v>
+      </c>
+      <c r="G21" s="17">
+        <v>0.17</v>
+      </c>
+      <c r="J21" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="K21" s="36">
+        <f>IF($J$18=$A$20,$J$12*$D$20,IF($J$18=$A$21,$J$12*$D$21,IF($J$18=$A$22,$J$12*$D$22,IF($J$18=$A$23,$J$12*$D$23,IF($J$18=$A$24,$J$12*$D$24,0)))))</f>
+        <v>2.9966538461538461E-2</v>
+      </c>
+      <c r="L21" s="36"/>
+      <c r="M21" s="29">
+        <f t="shared" si="0"/>
+        <v>599.33076923076919</v>
+      </c>
+    </row>
+    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A22" s="16" t="s">
+        <v>11</v>
+      </c>
+      <c r="B22" s="17">
+        <v>0.24</v>
+      </c>
+      <c r="C22" s="17">
+        <v>0.15</v>
+      </c>
+      <c r="D22" s="17">
+        <v>0.1492</v>
+      </c>
+      <c r="E22" s="17">
+        <v>3.2300000000000002E-2</v>
+      </c>
+      <c r="F22" s="17">
+        <v>0.23849999999999999</v>
+      </c>
+      <c r="G22" s="17">
+        <v>0.19</v>
+      </c>
+      <c r="J22" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="K22" s="36">
+        <f>IF($J$18=$A$20,$J$12*$E$20,IF($J$18=$A$21,$J$12*$E$21,IF($J$18=$A$22,$J$12*$E$22,IF($J$18=$A$23,$J$12*$E$23,IF($J$18=$A$24,$J$12*$E$24,0)))))</f>
+        <v>6.4921153846153844E-3</v>
+      </c>
+      <c r="L22" s="36"/>
+      <c r="M22" s="29">
+        <f t="shared" si="0"/>
+        <v>129.84230769230768</v>
+      </c>
+    </row>
+    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A23" s="16" t="s">
+        <v>13</v>
+      </c>
+      <c r="B23" s="17">
+        <v>0.21</v>
+      </c>
+      <c r="C23" s="17">
+        <v>0.15</v>
+      </c>
+      <c r="D23" s="17">
+        <v>0.15740000000000001</v>
+      </c>
+      <c r="E23" s="17">
+        <v>3.4099999999999998E-2</v>
+      </c>
+      <c r="F23" s="17">
+        <v>0.23849999999999999</v>
+      </c>
+      <c r="G23" s="17">
+        <v>0.21</v>
+      </c>
+      <c r="J23" s="27" t="s">
+        <v>43</v>
+      </c>
+      <c r="K23" s="36">
+        <f>IF($J$18=$A$20,$J$12*$F$20,IF($J$18=$A$21,$J$12*$F$21,IF($J$18=$A$22,$J$12*$F$22,IF($J$18=$A$23,$J$12*$F$23,IF($J$18=$A$24,$J$12*$F$24,0)))))</f>
+        <v>4.5406730769230762E-2</v>
+      </c>
+      <c r="L23" s="36"/>
+      <c r="M23" s="29">
+        <f t="shared" si="0"/>
+        <v>908.13461538461524</v>
+      </c>
+    </row>
+    <row r="24" spans="1:13" ht="13.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24" s="16" t="s">
+        <v>15</v>
+      </c>
+      <c r="B24" s="17">
+        <v>0.23</v>
+      </c>
+      <c r="C24" s="17">
+        <v>0.125</v>
+      </c>
+      <c r="D24" s="17">
+        <v>0.14099999999999999</v>
+      </c>
+      <c r="E24" s="17">
+        <v>3.0499999999999999E-2</v>
+      </c>
+      <c r="F24" s="17">
+        <v>0.23849999999999999</v>
+      </c>
+      <c r="G24" s="17">
+        <v>0.23499999999999999</v>
+      </c>
+      <c r="J24" s="30" t="s">
+        <v>49</v>
+      </c>
+      <c r="K24" s="39">
+        <f>IF($J$18=$A$20,$J$12*$G$20,IF($J$18=$A$21,$J$12*$G$21,IF($J$18=$A$22,$J$12*$G$22,IF($J$18=$A$23,$J$12*$G$23,IF($J$18=$A$24,$J$12*$G$24,0)))))</f>
+        <v>3.9980769230769229E-2</v>
+      </c>
+      <c r="L24" s="39"/>
+      <c r="M24" s="31">
+        <f t="shared" si="0"/>
+        <v>799.61538461538464</v>
+      </c>
+    </row>
+    <row r="25" spans="1:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B25" s="17">
+        <v>0.35</v>
+      </c>
+      <c r="C25" s="17">
+        <v>0.155</v>
+      </c>
+      <c r="D25" s="17">
+        <v>0.16439999999999999</v>
+      </c>
+      <c r="E25" s="17">
+        <v>3.56E-2</v>
+      </c>
+      <c r="F25" s="17">
+        <v>0.29499999999999998</v>
+      </c>
+      <c r="G25" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="J25" s="32" t="s">
+        <v>68</v>
+      </c>
+      <c r="K25" s="38">
+        <f>SUM(K19:L24)</f>
+        <v>0.19038461538461537</v>
+      </c>
+      <c r="L25" s="38"/>
+      <c r="M25" s="33">
+        <f>SUM(M19:M24)</f>
+        <v>3807.6923076923076</v>
+      </c>
+    </row>
+    <row r="26" spans="1:13" ht="13.5" customHeight="1" x14ac:dyDescent="0.25"/>
+  </sheetData>
+  <mergeCells count="23">
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="A18:A19"/>
+    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="K18:L18"/>
+    <mergeCell ref="K19:L19"/>
+    <mergeCell ref="K20:L20"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="E12:E13"/>
+    <mergeCell ref="J12:J13"/>
+    <mergeCell ref="F13:I13"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="F15:G16"/>
+    <mergeCell ref="J17:M17"/>
+    <mergeCell ref="I2:J2"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="E6:E7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="F9:F10"/>
+  </mergeCells>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>